<commit_message>
fix the error prompt in m12, fix the pricing detection issue
</commit_message>
<xml_diff>
--- a/src/scraping/data/test_data/initial_url.xlsx
+++ b/src/scraping/data/test_data/initial_url.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\programming\competitor_product_search\src\scraping\data\test_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23A4EB04-47D3-4810-9EFD-69A53AAF1385}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E31EA572-07E3-4682-BE0F-FDE28FEB9185}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="3795" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="75300" yWindow="6120" windowWidth="16425" windowHeight="14010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -75,9 +75,6 @@
     <t>argos.co.uk</t>
   </si>
   <si>
-    <t>https://www.argos.co.uk/product/8747437</t>
-  </si>
-  <si>
     <t>https://www.argos.co.uk/product/7726844</t>
   </si>
   <si>
@@ -135,6 +132,10 @@
   </si>
   <si>
     <t>unavailable</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.argos.co.uk/product/8747437</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -483,7 +484,7 @@
   <dimension ref="A1:C23"/>
   <sheetFormatPr defaultRowHeight="14.1" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="2" max="2" width="14.19921875" customWidth="1"/>
+    <col min="2" max="2" width="24.94921875" customWidth="1"/>
     <col min="3" max="3" width="11.09765625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -500,10 +501,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C2" t="s">
         <v>13</v>
@@ -511,7 +512,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>2</v>
@@ -522,7 +523,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>3</v>
@@ -547,7 +548,7 @@
         <v>9</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C6" t="s">
         <v>13</v>
@@ -566,7 +567,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>6</v>
@@ -602,7 +603,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C11" t="s">
         <v>15</v>
@@ -613,7 +614,7 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>16</v>
+        <v>34</v>
       </c>
       <c r="C12" t="s">
         <v>15</v>
@@ -624,7 +625,7 @@
         <v>9</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C13" t="s">
         <v>15</v>
@@ -635,7 +636,7 @@
         <v>10</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C14" t="s">
         <v>15</v>
@@ -646,7 +647,7 @@
         <v>9</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C15" t="s">
         <v>15</v>
@@ -657,7 +658,7 @@
         <v>11</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C16" t="s">
         <v>15</v>
@@ -668,7 +669,7 @@
         <v>11</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C17" t="s">
         <v>15</v>
@@ -676,13 +677,13 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A18" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B18" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C18" t="s">
         <v>21</v>
-      </c>
-      <c r="C18" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.5">
@@ -690,32 +691,32 @@
         <v>9</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A20" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C20" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A21" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C21" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.5">
@@ -723,10 +724,10 @@
         <v>9</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.5">
@@ -734,10 +735,10 @@
         <v>10</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C23" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>